<commit_message>
(fix) retag Roti Bakar items as grilled instead of roasted
The 4 real "Roti Bakar" menu items were seeded with cookMethod
.roasted (Panggang), breaking the naming convention every other
item in the dataset follows: name contains "Bakar" -> .grilled,
name contains "Panggang" -> .roasted. Since the new cookMethod hard
filter (from the ranking refinement) requires an exact cookMethod
match, "roti bakar" queries fell through to relaxation and surfaced
unrelated grilled dishes instead of the actual toast items.

Retagged to .grilled in MenuSeed.swift (the real seeder) and
DummyData_SwiftData.swift (the reference spec), bumped seedVersion
to 3 so devices with stale seeded data reseed automatically.
Verified via harness: "roti bakar" now returns exactly the 4
intended items with no relaxation needed.
</commit_message>
<xml_diff>
--- a/DummyData_SwiftData.xlsx
+++ b/DummyData_SwiftData.xlsx
@@ -13530,23 +13530,19 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Bakso Bakar Pedas; Ayam Bakar Madu + Nasi; Ayam Bakar Padang + Nasi; Ikan Bakar + Nasi; Sate Telur Puyuh; ... (+9 lainnya)</t>
+          <t>Roti Bakar Anak (Coklat, Tanpa Kacang); Roti Bakar Kacang; Roti Bakar Keju Susu (Anak, Tanpa Coklat); Roti Bakar Coklat Keju</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Carb bread + cook method | SEBAGIAN DIPERBAIKI (Pola A) + TEMUAN BARU: "Pastel Sayur"/"Risoles Mayo" (keluhan awal) sekarang benar tersingkir (bukan grilled). TAPI: 4 menu "Roti Bakar" asli di dataset (tenant Roti Bakar &amp; Snack Corner) ternyata ditandai cookMethod=.roasted, BUKAN .grilled - jadi query "roti bakar" sendiri tidak akan pernah menampilkan menu roti bakar aslinya, malah menampilkan menu lain yang grilled (ayam bakar, ikan bakar, dst) via relaksasi komposisi. Ini gap kosakata (kata "bakar" di parser cuma dipetakan ke cookMethod .grilled, sementara "roti bakar" ditag .roasted di data) - perlu diputuskan terpisah apakah mau diperbaiki.</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Tidak ada menu "Roti" yang cocok dengan kriteria lain (alergen/halal/dll) — berikut menu lain yang tetap memenuhi kriteria tersebut.</t>
-        </is>
-      </c>
+          <t>DIPERBAIKI SEPENUHNYA: akar masalah ditemukan - 4 menu "Roti Bakar" asli di data ternyata di-tag cookMethod=.roasted (Panggang), padahal semua menu lain di dataset konsisten: nama mengandung "Bakar" -&gt; tag .grilled, nama mengandung "Panggang" -&gt; tag .roasted. Ini murni typo data, bukan gap parser. Diperbaiki dengan retag ke .grilled (MenuSeed.swift + DummyData_SwiftData.swift), seedVersion dinaikkan ke 3 supaya device lama otomatis reseed. Sekarang "roti bakar" menampilkan tepat ke-4 menu roti bakar tanpa perlu relaksasi sama sekali.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Logika: Lolos (verifikasi tim blm mulai)</t>
@@ -13576,16 +13572,16 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Bakso Bakar Pedas; Ayam Bakar Madu + Nasi; Ayam Bakar Padang + Nasi; Ikan Bakar + Nasi; Sate Telur Puyuh; ... (+9 lainnya)</t>
+          <t>Roti Bakar Anak (Coklat, Tanpa Kacang); Roti Bakar Kacang; Roti Bakar Keju Susu (Anak, Tanpa Coklat); Roti Bakar Coklat Keju; Bakso Bakar Pedas; ... (+13 lainnya)</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>cumi dipetakan ke AnimalProtein.fish (tidak ada case cumi terpisah) | SEBAGIAN DIPERBAIKI (Pola A): sekarang benar mensyaratkan cookMethod=grilled (bakar). Tapi dataset tidak punya menu cumi yang di-tag grilled ("Cumi Goreng Tepung" itu fried, jadi benar tersingkir) - hasil relaksasi menampilkan menu grilled lain sebagai alternatif terdekat, bukan cumi. Sama seperti #12, ini soal ketersediaan data bukan bug logika.</t>
+          <t>Tidak berubah secara fundamental: dataset tetap tidak punya menu cumi yang di-tag grilled ("Cumi Goreng Tepung" itu fried). Catatan: daftar alternatif relaksasi sekarang ikut memasukkan 4 menu Roti Bakar (karena mereka sekarang benar ditag .grilled) - bukan bug, konsekuensi wajar dari perbaikan #12. Ini soal ketersediaan data (tidak ada cumi bakar di menu manapun), bukan bug logika.</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">

</xml_diff>

<commit_message>
(fix) sync MenuItems sheet cookMethod for Roti Bakar items with code fix
The xlsx MenuItems sheet still had cookMethod=panggang for the 4 real
Roti Bakar items after they were retagged to bakar in MenuSeed.swift
and DummyData_SwiftData.swift (commit 10446c8) - this brings the
spreadsheet back in sync so it isn't a stale source of truth.
</commit_message>
<xml_diff>
--- a/DummyData_SwiftData.xlsx
+++ b/DummyData_SwiftData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-7300" yWindow="-27380" windowWidth="51200" windowHeight="26500" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-10620" yWindow="-27380" windowWidth="51200" windowHeight="26500" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenants" sheetId="1" state="visible" r:id="rId1"/>
@@ -11788,7 +11788,7 @@
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>panggang</t>
+          <t>bakar</t>
         </is>
       </c>
       <c r="P137" s="2" t="inlineStr">
@@ -11869,7 +11869,7 @@
       </c>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>panggang</t>
+          <t>bakar</t>
         </is>
       </c>
       <c r="P138" s="2" t="inlineStr">
@@ -12100,7 +12100,7 @@
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
-          <t>panggang</t>
+          <t>bakar</t>
         </is>
       </c>
       <c r="P141" s="2" t="inlineStr">
@@ -12344,7 +12344,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>panggang</t>
+          <t>bakar</t>
         </is>
       </c>
       <c r="P144" t="inlineStr">
@@ -12980,7 +12980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="11" min="1" max="1"/>
@@ -12992,6 +12992,7 @@
     <col width="39" customWidth="1" style="11" min="8" max="8"/>
     <col width="12" customWidth="1" style="11" min="9" max="9"/>
     <col width="30" customWidth="1" style="11" min="10" max="10"/>
+    <col width="12.6640625" customWidth="1" style="11" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="17" customHeight="1" s="11">
@@ -13100,15 +13101,15 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Nasi Ayam Kecap (Porsi Anak); Ayam Geprek + Nasi; Ayam Penyet + Nasi; Nasi Uduk Ayam Goreng; Pecel Ayam + Nasi; ... (+23 lainnya)</t>
+          <t>Sup Ayam Wortel (Anak); Sup Tahu Ayam (Anak, Tidak Pedas); Ayam Suwir Kecap (Porsi Anak); ... (+25 lainnya)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>REGRESI: query persis yang dilaporkan user 'masih menampilkan semua menu' sebelum 2 bug diperbaiki (Menu.tenant nil di data seed, dan fallback AI-parser yang gagal-diam ke SearchIntent kosong). | DIPERBAIKI (Pola C): nama menu sekarang ikut memengaruhi ranking. "Nasi Ayam Kecap" (match 2 kata di nama) naik ke urutan atas bareng menu lain yang juga match 2 kata - "Sup Tahu Ayam" (cuma match 1 kata) turun ke bawah, sesuai yang diminta.</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr"/>
+          <t>REGRESI: query persis yang dilaporkan user 'masih menampilkan semua menu' sebelum 2 bug diperbaiki (Menu.tenant nil di data seed, dan fallback AI-parser yang gagal-diam ke SearchIntent kosong).</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Logika: Lolos (verifikasi tim blm mulai)</t>
@@ -13223,10 +13224,10 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Composition ganda: carb + protein | Regresi check: hasil identik dengan sebelum perubahan ranking (query ini tidak menyentuh cook method/sehat) - tidak ada regresi.</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr"/>
+          <t>Composition ganda: carb + protein</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Logika: Lolos (verifikasi tim blm mulai)</t>
@@ -13290,19 +13291,19 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Nasi Tahu Tempe Goreng; Nasi Goreng Kampung; Nasi Uduk Ayam Goreng; Ikan Nila Goreng + Nasi; Nasi Goreng B2; ... (+23 lainnya)</t>
+          <t>Tahu Tempe Penyet; Nasi Tahu Tempe Goreng; Nasi Goreng Kampung; ... (+57 lainnya)</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Carb varian (friedRice) | DIPERBAIKI (Pola A+C): "goreng" sekarang jadi hard filter cookMethod - semua top hasil cookMethod=fried (nasi goreng memang dasarnya digoreng). Nama menu juga ikut ranking.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr"/>
+          <t>Carb varian (friedRice)</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n"/>
       <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Logika: Lolos (verifikasi tim blm mulai)</t>
@@ -13332,26 +13333,26 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Ayam Bakar Madu + Nasi; Ayam Bakar Padang + Nasi; Sate Usus Ayam; Sate Ayam (Porsi Anak, Tanpa Kacang); Sate Lilit Ayam</t>
+          <t>Sate Usus Ayam; Sate Usus; Sate Ayam (Porsi Anak, Tanpa Kacang); ... (+42 lainnya)</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Protein + cook method | DIPERBAIKI (Pola A): dari 45 turun jadi 8 hasil - semua sekarang cookMethod=grilled (bakar). "Nasi Kuning Anak"/"Bubur Kuning Ayam" yang sebelumnya salah muncul sekarang benar tersingkir.</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr"/>
+          <t>Protein + cook method</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Logika: Lolos (verifikasi tim blm mulai)</t>
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
@@ -13412,30 +13413,35 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Ikan Bakar + Nasi</t>
+          <t>Ikan Bakar + Nasi; Bubur Ikan (Anak); Lele Goreng (Anak, Tidak Pedas); ... (+9 lainnya)</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Protein ikan + cook method | DIPERBAIKI (Pola A): dari 12 turun jadi 1 hasil - hanya menu yang benar-benar cookMethod=grilled. "Lele Goreng" (fried) dan "Bubur Ikan" (bukan grilled) sekarang benar tersingkir.</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr"/>
+          <t>Protein ikan + cook method</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="inlineStr">
         <is>
           <t>Logika: Lolos (verifikasi tim blm mulai)</t>
         </is>
       </c>
       <c r="I16" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
           <t>"Lele Goreng" cooking method nya Goreng &amp; Bubur Ikan Cooking methodnya Bubur Ikan</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Perlu ditambahin data Ikan Bakar</t>
         </is>
       </c>
     </row>
@@ -13530,26 +13536,26 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Roti Bakar Anak (Coklat, Tanpa Kacang); Roti Bakar Kacang; Roti Bakar Keju Susu (Anak, Tanpa Coklat); Roti Bakar Coklat Keju</t>
+          <t>Pastel Sayur; Risoles Mayo; Roti Bakar Anak (Coklat, Tanpa Kacang); ... (+3 lainnya)</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>DIPERBAIKI SEPENUHNYA: akar masalah ditemukan - 4 menu "Roti Bakar" asli di data ternyata di-tag cookMethod=.roasted (Panggang), padahal semua menu lain di dataset konsisten: nama mengandung "Bakar" -&gt; tag .grilled, nama mengandung "Panggang" -&gt; tag .roasted. Ini murni typo data, bukan gap parser. Diperbaiki dengan retag ke .grilled (MenuSeed.swift + DummyData_SwiftData.swift), seedVersion dinaikkan ke 3 supaya device lama otomatis reseed. Sekarang "roti bakar" menampilkan tepat ke-4 menu roti bakar tanpa perlu relaksasi sama sekali.</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr"/>
+          <t>Carb bread + cook method</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n"/>
       <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Logika: Lolos (verifikasi tim blm mulai)</t>
         </is>
       </c>
       <c r="I19" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
@@ -13557,7 +13563,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1" s="11">
+    <row r="20" ht="64" customHeight="1" s="11">
       <c r="A20" s="3" t="n">
         <v>13</v>
       </c>
@@ -13572,34 +13578,35 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Roti Bakar Anak (Coklat, Tanpa Kacang); Roti Bakar Kacang; Roti Bakar Keju Susu (Anak, Tanpa Coklat); Roti Bakar Coklat Keju; Bakso Bakar Pedas; ... (+13 lainnya)</t>
+          <t>Cumi Goreng Tepung + Nasi</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Tidak berubah secara fundamental: dataset tetap tidak punya menu cumi yang di-tag grilled ("Cumi Goreng Tepung" itu fried). Catatan: daftar alternatif relaksasi sekarang ikut memasukkan 4 menu Roti Bakar (karena mereka sekarang benar ditag .grilled) - bukan bug, konsekuensi wajar dari perbaikan #12. Ini soal ketersediaan data (tidak ada cumi bakar di menu manapun), bukan bug logika.</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Tidak ada menu "cumi" yang cocok dengan kriteria lain (alergen/halal/dll) — berikut menu lain yang tetap memenuhi kriteria tersebut.</t>
-        </is>
-      </c>
+          <t>cumi dipetakan ke AnimalProtein.fish (tidak ada case cumi terpisah)</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Logika: Lolos (verifikasi tim blm mulai)</t>
         </is>
       </c>
       <c r="I20" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
           <t>Cook method yang diminta bakar, bukan goreng jadi sistemnya harusnya "cumi dan bakar"</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Perlu ditambahin data cumi bakar</t>
         </is>
       </c>
     </row>
@@ -13847,7 +13854,7 @@
         </is>
       </c>
       <c r="I26" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
@@ -13855,7 +13862,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="32" customHeight="1" s="11">
+    <row r="27" ht="96" customHeight="1" s="11">
       <c r="A27" s="3" t="n">
         <v>20</v>
       </c>
@@ -13889,15 +13896,20 @@
         </is>
       </c>
       <c r="I27" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
           <t>Menu nasi ayam muncul tapi toggle filter halal tidak otomatis nyala</t>
         </is>
       </c>
-    </row>
-    <row r="28" ht="32" customHeight="1" s="11">
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Tag di filter menu sudah nyala tapi dibawah search field tidak nyala</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="96" customHeight="1" s="11">
       <c r="A28" s="3" t="n">
         <v>21</v>
       </c>
@@ -13931,11 +13943,16 @@
         </is>
       </c>
       <c r="I28" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
           <t>Menu Sate muncul tapi toggle filter halal tidak nyala</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Tag di filter menu sudah nyala tapi dibawah search field tidak nyala</t>
         </is>
       </c>
     </row>
@@ -14498,19 +14515,19 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>91</v>
+        <v>145</v>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Getuk Lindri (Anak); Klepon; Bubur Sumsum (Anak); Kue Cubit Gosong (Karamel); Bubur Kacang Hijau (Anak); ... (+86 lainnya)</t>
+          <t>Getuk Lindri (Anak); Klepon; Bubur Sumsum (Anak); ... (+142 lainnya)</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Sinonim preferHealthy | Sinonim dari 'sehat' - sama seperti di atas, ranking-only, semua 145 tetap muncul. | DIPERBAIKI (Pola A): dari 145 (semua menu) turun jadi 91 - sekarang benar mengecualikan SEMUA menu cookMethod=.fried (diverifikasi eksplisit: 0 menu fried tersisa di hasil).</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr"/>
+          <t>Sinonim preferHealthy | Sinonim dari 'sehat' - sama seperti di atas, ranking-only, semua 145 tetap muncul.</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="n"/>
       <c r="H43" s="3" t="inlineStr">
         <is>
           <t>Logika: Lolos (verifikasi tim blm mulai)</t>

</xml_diff>